<commit_message>
LTBU changed, LTCH added
</commit_message>
<xml_diff>
--- a/lt_aerodromes.xlsx
+++ b/lt_aerodromes.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\website\aip downloader\AIP_downloader_LT\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ibosoft\diger-github-repolari\Index-of-Turkiye-Aerodromes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED6EB46-043F-4327-AE49-01956736296F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EFC669A-12DE-41E4-A8CC-4A075B47FA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CFEF53A2-6721-40FC-85FC-2D83DAB71C05}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{CFEF53A2-6721-40FC-85FC-2D83DAB71C05}"/>
   </bookViews>
   <sheets>
     <sheet name="Aerodromes" sheetId="2" r:id="rId1"/>
     <sheet name="info" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="DışVeri_1" localSheetId="0" hidden="1">Aerodromes!$A$1:$G$88</definedName>
+    <definedName name="DışVeri_1" localSheetId="0" hidden="1">Aerodromes!$A$1:$G$89</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="263">
   <si>
     <t>S - N - P - M</t>
   </si>
@@ -728,9 +728,6 @@
     <t>MANİSA - Akhisar</t>
   </si>
   <si>
-    <t>TEKİRDAĞ - Çorlu</t>
-  </si>
-  <si>
     <t>BODRUM - IMSIK</t>
   </si>
   <si>
@@ -830,7 +827,19 @@
     <t>RİZE - ARTVİN</t>
   </si>
   <si>
-    <t>IboSoft - rev.1</t>
+    <t>TEKİRDAĞ - Çorlu Atatürk</t>
+  </si>
+  <si>
+    <t>LTCH</t>
+  </si>
+  <si>
+    <t>ŞANLIURFA</t>
+  </si>
+  <si>
+    <t>SFQ</t>
+  </si>
+  <si>
+    <t>IboSoft - rev.1.2</t>
   </si>
 </sst>
 </file>
@@ -874,11 +883,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -931,10 +941,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3A216019-EDC6-4FF1-91EC-0BBBA30E30D2}" name="Aerodromes" displayName="Aerodromes" ref="A1:G88" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:G88" xr:uid="{3A216019-EDC6-4FF1-91EC-0BBBA30E30D2}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G88">
-    <sortCondition ref="B1:B88"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3A216019-EDC6-4FF1-91EC-0BBBA30E30D2}" name="Aerodromes" displayName="Aerodromes" ref="A1:G89" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:G89" xr:uid="{3A216019-EDC6-4FF1-91EC-0BBBA30E30D2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G89">
+    <sortCondition ref="B1:B89"/>
   </sortState>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{D918F25B-48AD-4198-8F61-5C1BFA5F856E}" uniqueName="1" name="Name" queryTableFieldId="1" dataDxfId="3"/>
@@ -1246,7 +1256,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0371283C-4A27-450C-9EFC-AC4555602BE3}">
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.7109375" customWidth="1"/>
@@ -1274,7 +1284,7 @@
         <v>10</v>
       </c>
       <c r="F1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G1" t="s">
         <v>12</v>
@@ -1314,10 +1324,10 @@
         <v>132</v>
       </c>
       <c r="E3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G3" t="s">
         <v>0</v>
@@ -1340,7 +1350,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G4" t="s">
         <v>6</v>
@@ -1360,7 +1370,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G5" t="s">
         <v>6</v>
@@ -1380,10 +1390,10 @@
         <v>132</v>
       </c>
       <c r="E6" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G6" t="s">
         <v>0</v>
@@ -1406,7 +1416,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G7" t="s">
         <v>6</v>
@@ -1429,7 +1439,7 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G8" t="s">
         <v>6</v>
@@ -1449,10 +1459,10 @@
         <v>132</v>
       </c>
       <c r="E9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G9" t="s">
         <v>0</v>
@@ -1472,10 +1482,10 @@
         <v>132</v>
       </c>
       <c r="E10" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F10" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G10" t="s">
         <v>0</v>
@@ -1495,10 +1505,10 @@
         <v>132</v>
       </c>
       <c r="E11" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F11" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G11" t="s">
         <v>0</v>
@@ -1518,10 +1528,10 @@
         <v>132</v>
       </c>
       <c r="E12" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F12" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G12" t="s">
         <v>0</v>
@@ -1529,7 +1539,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B13" t="s">
         <v>96</v>
@@ -1541,7 +1551,7 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G13" t="s">
         <v>6</v>
@@ -1561,10 +1571,10 @@
         <v>132</v>
       </c>
       <c r="E14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G14" t="s">
         <v>0</v>
@@ -1584,10 +1594,10 @@
         <v>132</v>
       </c>
       <c r="E15" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F15" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G15" t="s">
         <v>0</v>
@@ -1607,10 +1617,10 @@
         <v>132</v>
       </c>
       <c r="E16" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F16" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G16" t="s">
         <v>0</v>
@@ -1630,10 +1640,10 @@
         <v>132</v>
       </c>
       <c r="E17" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F17" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G17" t="s">
         <v>0</v>
@@ -1653,10 +1663,10 @@
         <v>132</v>
       </c>
       <c r="E18" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F18" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G18" t="s">
         <v>0</v>
@@ -1676,7 +1686,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G19" t="s">
         <v>6</v>
@@ -1696,10 +1706,10 @@
         <v>132</v>
       </c>
       <c r="E20" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G20" t="s">
         <v>0</v>
@@ -1719,10 +1729,10 @@
         <v>132</v>
       </c>
       <c r="E21" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F21" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G21" t="s">
         <v>0</v>
@@ -1742,10 +1752,10 @@
         <v>132</v>
       </c>
       <c r="E22" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F22" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G22" t="s">
         <v>0</v>
@@ -1765,10 +1775,10 @@
         <v>132</v>
       </c>
       <c r="E23" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F23" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G23" t="s">
         <v>0</v>
@@ -1791,7 +1801,7 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G24" t="s">
         <v>2</v>
@@ -1814,7 +1824,7 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G25" t="s">
         <v>0</v>
@@ -1837,7 +1847,7 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G26" t="s">
         <v>7</v>
@@ -1857,10 +1867,10 @@
         <v>132</v>
       </c>
       <c r="E27" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F27" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G27" t="s">
         <v>0</v>
@@ -1883,7 +1893,7 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G28" t="s">
         <v>6</v>
@@ -1903,10 +1913,10 @@
         <v>132</v>
       </c>
       <c r="E29" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F29" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G29" t="s">
         <v>0</v>
@@ -1949,7 +1959,7 @@
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G31" t="s">
         <v>6</v>
@@ -1989,10 +1999,10 @@
         <v>132</v>
       </c>
       <c r="E33" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F33" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G33" t="s">
         <v>0</v>
@@ -2032,10 +2042,10 @@
         <v>132</v>
       </c>
       <c r="E35" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F35" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G35" t="s">
         <v>0</v>
@@ -2055,10 +2065,10 @@
         <v>132</v>
       </c>
       <c r="E36" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F36" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G36" t="s">
         <v>0</v>
@@ -2078,10 +2088,10 @@
         <v>132</v>
       </c>
       <c r="E37" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F37" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G37" t="s">
         <v>0</v>
@@ -2101,7 +2111,7 @@
         <v>1</v>
       </c>
       <c r="F38" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G38" t="s">
         <v>6</v>
@@ -2109,7 +2119,7 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>225</v>
+        <v>258</v>
       </c>
       <c r="B39" t="s">
         <v>73</v>
@@ -2121,10 +2131,10 @@
         <v>132</v>
       </c>
       <c r="E39" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F39" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G39" t="s">
         <v>0</v>
@@ -2132,7 +2142,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B40" t="s">
         <v>86</v>
@@ -2147,7 +2157,7 @@
         <v>1</v>
       </c>
       <c r="F40" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G40" t="s">
         <v>6</v>
@@ -2155,7 +2165,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B41" t="s">
         <v>47</v>
@@ -2175,7 +2185,7 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B42" t="s">
         <v>90</v>
@@ -2195,7 +2205,7 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B43" t="s">
         <v>38</v>
@@ -2207,10 +2217,10 @@
         <v>132</v>
       </c>
       <c r="E43" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F43" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G43" t="s">
         <v>3</v>
@@ -2230,10 +2240,10 @@
         <v>132</v>
       </c>
       <c r="E44" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F44" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G44" t="s">
         <v>0</v>
@@ -2253,10 +2263,10 @@
         <v>132</v>
       </c>
       <c r="E45" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F45" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G45" t="s">
         <v>0</v>
@@ -2264,7 +2274,7 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B46" t="s">
         <v>64</v>
@@ -2276,10 +2286,10 @@
         <v>132</v>
       </c>
       <c r="E46" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F46" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G46" t="s">
         <v>0</v>
@@ -2299,10 +2309,10 @@
         <v>132</v>
       </c>
       <c r="E47" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F47" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G47" t="s">
         <v>0</v>
@@ -2310,7 +2320,7 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B48" t="s">
         <v>36</v>
@@ -2322,10 +2332,10 @@
         <v>132</v>
       </c>
       <c r="E48" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F48" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G48" t="s">
         <v>0</v>
@@ -2345,10 +2355,10 @@
         <v>132</v>
       </c>
       <c r="E49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G49" t="s">
         <v>0</v>
@@ -2368,10 +2378,10 @@
         <v>132</v>
       </c>
       <c r="E50" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G50" t="s">
         <v>0</v>
@@ -2391,56 +2401,47 @@
         <v>132</v>
       </c>
       <c r="E51" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F51" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G51" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>231</v>
+      <c r="A52" s="2" t="s">
+        <v>260</v>
       </c>
       <c r="B52" t="s">
-        <v>77</v>
+        <v>259</v>
       </c>
       <c r="C52" t="s">
-        <v>173</v>
-      </c>
-      <c r="D52" t="s">
-        <v>132</v>
-      </c>
-      <c r="E52" t="s">
-        <v>251</v>
-      </c>
-      <c r="F52" t="s">
-        <v>250</v>
-      </c>
-      <c r="G52" t="s">
-        <v>0</v>
-      </c>
+        <v>261</v>
+      </c>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>16</v>
+        <v>230</v>
       </c>
       <c r="B53" t="s">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="C53" t="s">
-        <v>143</v>
+        <v>173</v>
       </c>
       <c r="D53" t="s">
         <v>132</v>
       </c>
       <c r="E53" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F53" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G53" t="s">
         <v>0</v>
@@ -2448,22 +2449,22 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>232</v>
+        <v>16</v>
       </c>
       <c r="B54" t="s">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="C54" t="s">
-        <v>185</v>
+        <v>143</v>
       </c>
       <c r="D54" t="s">
         <v>132</v>
       </c>
       <c r="E54" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F54" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G54" t="s">
         <v>0</v>
@@ -2471,22 +2472,22 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>118</v>
+        <v>231</v>
       </c>
       <c r="B55" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C55" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D55" t="s">
         <v>132</v>
       </c>
       <c r="E55" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F55" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G55" t="s">
         <v>0</v>
@@ -2494,22 +2495,22 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B56" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C56" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D56" t="s">
         <v>132</v>
       </c>
       <c r="E56" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F56" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G56" t="s">
         <v>0</v>
@@ -2517,22 +2518,22 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="B57" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C57" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D57" t="s">
         <v>132</v>
       </c>
       <c r="E57" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F57" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G57" t="s">
         <v>0</v>
@@ -2540,22 +2541,22 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>254</v>
+        <v>111</v>
       </c>
       <c r="B58" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="C58" t="s">
-        <v>149</v>
+        <v>188</v>
       </c>
       <c r="D58" t="s">
         <v>132</v>
       </c>
       <c r="E58" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F58" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G58" t="s">
         <v>0</v>
@@ -2563,22 +2564,22 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>14</v>
+        <v>253</v>
       </c>
       <c r="B59" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C59" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D59" t="s">
         <v>132</v>
       </c>
       <c r="E59" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F59" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G59" t="s">
         <v>0</v>
@@ -2586,22 +2587,22 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>233</v>
+        <v>14</v>
       </c>
       <c r="B60" t="s">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="C60" t="s">
-        <v>189</v>
+        <v>148</v>
       </c>
       <c r="D60" t="s">
         <v>132</v>
       </c>
       <c r="E60" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F60" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G60" t="s">
         <v>0</v>
@@ -2609,22 +2610,22 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B61" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="C61" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D61" t="s">
         <v>132</v>
       </c>
       <c r="E61" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F61" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G61" t="s">
         <v>0</v>
@@ -2632,22 +2633,22 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B62" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="C62" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D62" t="s">
         <v>132</v>
       </c>
       <c r="E62" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F62" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G62" t="s">
         <v>0</v>
@@ -2655,22 +2656,22 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>17</v>
+        <v>234</v>
       </c>
       <c r="B63" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C63" t="s">
-        <v>153</v>
+        <v>191</v>
       </c>
       <c r="D63" t="s">
         <v>132</v>
       </c>
       <c r="E63" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F63" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G63" t="s">
         <v>0</v>
@@ -2678,22 +2679,22 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>236</v>
+        <v>17</v>
       </c>
       <c r="B64" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="C64" t="s">
-        <v>192</v>
+        <v>153</v>
       </c>
       <c r="D64" t="s">
         <v>132</v>
       </c>
       <c r="E64" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F64" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G64" t="s">
         <v>0</v>
@@ -2701,22 +2702,22 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
       <c r="B65" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="C65" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D65" t="s">
         <v>132</v>
       </c>
       <c r="E65" t="s">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="F65" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G65" t="s">
         <v>0</v>
@@ -2724,22 +2725,22 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>110</v>
+        <v>254</v>
       </c>
       <c r="B66" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C66" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D66" t="s">
         <v>132</v>
       </c>
       <c r="E66" t="s">
-        <v>251</v>
+        <v>1</v>
       </c>
       <c r="F66" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G66" t="s">
         <v>0</v>
@@ -2747,22 +2748,22 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>136</v>
+        <v>110</v>
       </c>
       <c r="B67" t="s">
-        <v>135</v>
+        <v>43</v>
       </c>
       <c r="C67" t="s">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="D67" t="s">
         <v>132</v>
       </c>
       <c r="E67" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F67" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G67" t="s">
         <v>0</v>
@@ -2770,88 +2771,88 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>237</v>
+        <v>136</v>
       </c>
       <c r="B68" t="s">
-        <v>93</v>
+        <v>135</v>
+      </c>
+      <c r="C68" t="s">
+        <v>158</v>
       </c>
       <c r="D68" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E68" t="s">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="F68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G68" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
       <c r="B69" t="s">
-        <v>51</v>
-      </c>
-      <c r="C69" t="s">
-        <v>195</v>
+        <v>93</v>
       </c>
       <c r="D69" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E69" t="s">
         <v>1</v>
       </c>
       <c r="F69" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G69" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B70" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C70" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D70" t="s">
         <v>132</v>
       </c>
       <c r="E70" t="s">
-        <v>251</v>
+        <v>1</v>
       </c>
       <c r="F70" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G70" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="B71" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="C71" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D71" t="s">
         <v>132</v>
       </c>
       <c r="E71" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F71" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G71" t="s">
         <v>0</v>
@@ -2859,22 +2860,22 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B72" t="s">
-        <v>61</v>
+        <v>28</v>
       </c>
       <c r="C72" t="s">
-        <v>155</v>
+        <v>198</v>
       </c>
       <c r="D72" t="s">
         <v>132</v>
       </c>
       <c r="E72" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F72" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G72" t="s">
         <v>0</v>
@@ -2882,22 +2883,22 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B73" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="C73" t="s">
-        <v>199</v>
+        <v>155</v>
       </c>
       <c r="D73" t="s">
         <v>132</v>
       </c>
       <c r="E73" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F73" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G73" t="s">
         <v>0</v>
@@ -2905,88 +2906,88 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>239</v>
+      </c>
+      <c r="B74" t="s">
+        <v>40</v>
+      </c>
+      <c r="C74" t="s">
+        <v>199</v>
+      </c>
+      <c r="D74" t="s">
+        <v>132</v>
+      </c>
+      <c r="E74" t="s">
+        <v>250</v>
+      </c>
+      <c r="F74" t="s">
+        <v>249</v>
+      </c>
+      <c r="G74" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>240</v>
+      </c>
+      <c r="B75" t="s">
+        <v>66</v>
+      </c>
+      <c r="C75" t="s">
+        <v>200</v>
+      </c>
+      <c r="D75" t="s">
+        <v>132</v>
+      </c>
+      <c r="E75" t="s">
+        <v>250</v>
+      </c>
+      <c r="F75" t="s">
+        <v>249</v>
+      </c>
+      <c r="G75" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="B74" t="s">
-        <v>66</v>
-      </c>
-      <c r="C74" t="s">
-        <v>200</v>
-      </c>
-      <c r="D74" t="s">
-        <v>132</v>
-      </c>
-      <c r="E74" t="s">
-        <v>251</v>
-      </c>
-      <c r="F74" t="s">
-        <v>250</v>
-      </c>
-      <c r="G74" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="B75" t="s">
+      <c r="B76" t="s">
         <v>67</v>
       </c>
-      <c r="D75" t="s">
-        <v>132</v>
-      </c>
-      <c r="E75" t="s">
+      <c r="D76" t="s">
+        <v>132</v>
+      </c>
+      <c r="E76" t="s">
         <v>1</v>
       </c>
-      <c r="F75" t="s">
+      <c r="F76" t="s">
         <v>4</v>
       </c>
-      <c r="G75" t="s">
+      <c r="G76" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>243</v>
-      </c>
-      <c r="B76" t="s">
-        <v>49</v>
-      </c>
-      <c r="C76" t="s">
-        <v>201</v>
-      </c>
-      <c r="D76" t="s">
-        <v>132</v>
-      </c>
-      <c r="E76" t="s">
-        <v>251</v>
-      </c>
-      <c r="F76" t="s">
-        <v>250</v>
-      </c>
-      <c r="G76" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>109</v>
+        <v>242</v>
       </c>
       <c r="B77" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C77" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D77" t="s">
         <v>132</v>
       </c>
       <c r="E77" t="s">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="F77" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G77" t="s">
         <v>0</v>
@@ -2994,116 +2995,119 @@
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="B78" t="s">
-        <v>94</v>
+        <v>41</v>
+      </c>
+      <c r="C78" t="s">
+        <v>202</v>
       </c>
       <c r="D78" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E78" t="s">
         <v>1</v>
       </c>
       <c r="F78" t="s">
-        <v>4</v>
+        <v>249</v>
       </c>
       <c r="G78" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>244</v>
+        <v>126</v>
       </c>
       <c r="B79" t="s">
-        <v>48</v>
-      </c>
-      <c r="C79" t="s">
-        <v>196</v>
+        <v>94</v>
       </c>
       <c r="D79" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E79" t="s">
-        <v>251</v>
+        <v>1</v>
       </c>
       <c r="F79" t="s">
-        <v>250</v>
+        <v>4</v>
       </c>
       <c r="G79" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B80" t="s">
-        <v>89</v>
+        <v>48</v>
+      </c>
+      <c r="C80" t="s">
+        <v>196</v>
       </c>
       <c r="D80" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E80" t="s">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="F80" t="s">
-        <v>4</v>
+        <v>249</v>
       </c>
       <c r="G80" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="B81" t="s">
-        <v>65</v>
-      </c>
-      <c r="C81" t="s">
-        <v>203</v>
+        <v>89</v>
       </c>
       <c r="D81" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E81" t="s">
-        <v>251</v>
+        <v>1</v>
       </c>
       <c r="F81" t="s">
-        <v>250</v>
+        <v>4</v>
       </c>
       <c r="G81" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>246</v>
+        <v>257</v>
       </c>
       <c r="B82" t="s">
-        <v>99</v>
+        <v>65</v>
+      </c>
+      <c r="C82" t="s">
+        <v>203</v>
       </c>
       <c r="D82" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E82" t="s">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="F82" t="s">
-        <v>4</v>
+        <v>249</v>
       </c>
       <c r="G82" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B83" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D83" t="s">
         <v>134</v>
@@ -3120,10 +3124,10 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>18</v>
+        <v>246</v>
       </c>
       <c r="B84" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D84" t="s">
         <v>134</v>
@@ -3139,11 +3143,11 @@
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A85" s="1" t="s">
-        <v>248</v>
+      <c r="A85" t="s">
+        <v>18</v>
       </c>
       <c r="B85" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D85" t="s">
         <v>134</v>
@@ -3159,11 +3163,11 @@
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>249</v>
+      <c r="A86" s="1" t="s">
+        <v>247</v>
       </c>
       <c r="B86" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D86" t="s">
         <v>134</v>
@@ -3180,10 +3184,10 @@
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>129</v>
+        <v>248</v>
       </c>
       <c r="B87" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D87" t="s">
         <v>134</v>
@@ -3195,15 +3199,15 @@
         <v>4</v>
       </c>
       <c r="G87" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B88" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D88" t="s">
         <v>134</v>
@@ -3215,6 +3219,26 @@
         <v>4</v>
       </c>
       <c r="G88" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>130</v>
+      </c>
+      <c r="B89" t="s">
+        <v>105</v>
+      </c>
+      <c r="D89" t="s">
+        <v>134</v>
+      </c>
+      <c r="E89" t="s">
+        <v>1</v>
+      </c>
+      <c r="F89" t="s">
+        <v>4</v>
+      </c>
+      <c r="G89" t="s">
         <v>8</v>
       </c>
     </row>
@@ -3235,7 +3259,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>

</xml_diff>